<commit_message>
adicionada impressão e avaliação pediátrica
</commit_message>
<xml_diff>
--- a/img/modelo_input.xlsx
+++ b/img/modelo_input.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/431d7acb02e493d6/Documents/pre_automatizado/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/431d7acb02e493d6/Documents/pre_automatizado/img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B805C919-5F44-4844-A938-28124010C5C6}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5E4BA51-5A70-4CFD-9C9B-5A247825AFC7}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -427,7 +427,7 @@
       </c>
       <c r="C2" s="1">
         <f>VLOOKUP(A2,database!$A$1:$C$11,3,0)</f>
-        <v>32216</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -565,8 +565,8 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2">
-        <v>32216</v>
+      <c r="C2" s="1">
+        <v>46132</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -576,7 +576,7 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>35025</v>
       </c>
     </row>
@@ -587,7 +587,7 @@
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>36896</v>
       </c>
     </row>
@@ -598,7 +598,7 @@
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>33815</v>
       </c>
     </row>
@@ -609,7 +609,7 @@
       <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>30943</v>
       </c>
     </row>
@@ -620,7 +620,7 @@
       <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="1">
         <v>36292</v>
       </c>
     </row>
@@ -631,7 +631,7 @@
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>27817</v>
       </c>
     </row>
@@ -642,7 +642,7 @@
       <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="1">
         <v>34251</v>
       </c>
     </row>
@@ -653,7 +653,7 @@
       <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <v>32680</v>
       </c>
     </row>
@@ -664,7 +664,7 @@
       <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>35767</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualizacao das imagens para geracao
</commit_message>
<xml_diff>
--- a/img/modelo_input.xlsx
+++ b/img/modelo_input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/431d7acb02e493d6/Documents/pre_automatizado/img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5E4BA51-5A70-4CFD-9C9B-5A247825AFC7}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{971DCCA3-46BA-422B-A866-140066163AA7}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -419,7 +419,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>1234567</v>
       </c>
       <c r="B2" t="str">
         <f>VLOOKUP(A2,database!$A$1:$C$11,2,0)</f>
@@ -432,7 +432,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1234568</v>
       </c>
       <c r="B3" t="str">
         <f>VLOOKUP(A3,database!$A$1:$C$11,2,0)</f>
@@ -560,7 +560,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>1234567</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -571,7 +571,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1234568</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
melhorias sugeridas pela equipe
</commit_message>
<xml_diff>
--- a/img/modelo_input.xlsx
+++ b/img/modelo_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/431d7acb02e493d6/Documents/pre_automatizado/img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{971DCCA3-46BA-422B-A866-140066163AA7}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12DE284C-13BE-4D94-9CE1-E2D7F2FD54A2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -440,7 +440,7 @@
       </c>
       <c r="C3" s="1">
         <f>VLOOKUP(A3,database!$A$1:$C$11,3,0)</f>
-        <v>35025</v>
+        <v>20415</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -577,7 +577,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="1">
-        <v>35025</v>
+        <v>20415</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
adicão de turno e nome do médico, adição de cross e correção de layout sadt
</commit_message>
<xml_diff>
--- a/img/modelo_input.xlsx
+++ b/img/modelo_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/431d7acb02e493d6/Documents/pre_automatizado/img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12DE284C-13BE-4D94-9CE1-E2D7F2FD54A2}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="11_AD4D361C20488DEA4E38A04EE4DD75125BDEDD92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9222F423-64DA-4F8B-9C9C-2C194D2F292D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>Matrícula</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>Vanessa Cristina Santos</t>
+  </si>
+  <si>
+    <t>Teste Teste Teste</t>
   </si>
 </sst>
 </file>
@@ -129,10 +132,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -398,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" customWidth="1"/>
@@ -532,6 +531,17 @@
       <c r="C10" s="1">
         <f>VLOOKUP(A10,database!$A$1:$C$11,3,0)</f>
         <v>32680</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>999</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1">
+        <v>36161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>